<commit_message>
Update: ZİRAAT POS Temmuz 2026 daily gross amounts - correct data from user Excel
</commit_message>
<xml_diff>
--- a/ISIK_PETROL-ZIRAAT_POS-Gunluk_Brut-Temmuz2026.xlsx
+++ b/ISIK_PETROL-ZIRAAT_POS-Gunluk_Brut-Temmuz2026.xlsx
@@ -68,14 +68,10 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -442,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -462,323 +458,333 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>01.07.2026</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>0</v>
+      <c r="B2" s="2" t="n">
+        <v>338301.98</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>02.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>2113.82</v>
+      <c r="B3" s="2" t="n">
+        <v>225759.49</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>03.07.2026</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>31945.55</v>
+      <c r="B4" s="2" t="n">
+        <v>416049.6399999999</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>04.07.2026</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>41722.34</v>
+      <c r="B5" s="2" t="n">
+        <v>396190.33</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>05.07.2026</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
-        <v>75385.50999999999</v>
+      <c r="B6" s="2" t="n">
+        <v>355203.8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>06.07.2026</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>103514.87</v>
+      <c r="B7" s="2" t="n">
+        <v>294076.04</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>07.07.2026</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>1000</v>
+      <c r="B8" s="2" t="n">
+        <v>325567.8</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>08.07.2026</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>3537.92</v>
+      <c r="B9" s="2" t="n">
+        <v>379197.8700000001</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>09.07.2026</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
-        <v>27556.12</v>
+      <c r="B10" s="2" t="n">
+        <v>372869.04</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>10.07.2026</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>6514.03</v>
+      <c r="B11" s="2" t="n">
+        <v>318612.03</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>11.07.2026</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>3395.76</v>
+      <c r="B12" s="2" t="n">
+        <v>349301.96</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>12.07.2026</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
-        <v>495.05</v>
+      <c r="B13" s="2" t="n">
+        <v>380875.8100000001</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>13.07.2026</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
-        <v>2500</v>
+      <c r="B14" s="2" t="n">
+        <v>201828.23</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
-        <v>21910.52</v>
+      <c r="B15" s="2" t="n">
+        <v>203854.68</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>15.07.2026</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
-        <v>69750.25999999999</v>
+      <c r="B16" s="2" t="n">
+        <v>208477.19</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>16.07.2026</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
-        <v>62551.75</v>
+      <c r="B17" s="2" t="n">
+        <v>297138.79</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>17.07.2026</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
-        <v>148265.28</v>
+      <c r="B18" s="2" t="n">
+        <v>293177.15</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>18.07.2026</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
-        <v>5776.61</v>
+      <c r="B19" s="2" t="n">
+        <v>264097.5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>19.07.2026</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
-        <v>14070.55</v>
+      <c r="B20" s="2" t="n">
+        <v>315424.51</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>20.07.2026</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
-        <v>9600</v>
+      <c r="B21" s="2" t="n">
+        <v>206327.13</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>21.07.2026</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
-        <v>10474.65</v>
+      <c r="B22" s="2" t="n">
+        <v>308079.12</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>22.07.2026</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
-        <v>3200</v>
+      <c r="B23" s="2" t="n">
+        <v>253484.04</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>23.07.2026</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
-        <v>25221.14</v>
+      <c r="B24" s="2" t="n">
+        <v>307407.97</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>24.07.2026</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
-        <v>78164.12</v>
+      <c r="B25" s="2" t="n">
+        <v>464717.5699999999</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>25.07.2026</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
-        <v>123932.41</v>
+      <c r="B26" s="2" t="n">
+        <v>339722.67</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>26.07.2026</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
-        <v>165301.17</v>
+      <c r="B27" s="2" t="n">
+        <v>316778.91</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>27.07.2026</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
-        <v>12319.49</v>
+      <c r="B28" s="2" t="n">
+        <v>242373.85</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>28.07.2026</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
-        <v>22845.53</v>
+      <c r="B29" s="2" t="n">
+        <v>295067.15</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>29.07.2026</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
-        <v>28173.8</v>
+      <c r="B30" s="2" t="n">
+        <v>344899.62</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>30.07.2026</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
-        <v>23261.41</v>
+      <c r="B31" s="2" t="n">
+        <v>482419.0699999999</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>31.07.2026</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
-        <v>3150</v>
+      <c r="B32" s="2" t="n">
+        <v>393524.42</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TOPLAM</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>9890805.359999999</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B33" s="4">
-        <f>SUM(B2:B32)</f>
+      <c r="B34" s="4">
+        <f>SUM(B2:B33)</f>
         <v/>
       </c>
     </row>

</xml_diff>